<commit_message>
Add Lesson 1.5 confidence interval simulations on bakery data
</commit_message>
<xml_diff>
--- a/lesson-1-4-visualizing-distributions/bakery_distributions.xlsx
+++ b/lesson-1-4-visualizing-distributions/bakery_distributions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/johnko/northstar-coursework/module-01-foundations-of-analytics-and-statistics/lesson-1-4-visualizing-distributions/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{DCBF59D3-75A2-8540-887B-CCEEB3445491}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{00607A67-44D1-8F48-BD50-3F1E46CA2779}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="21000" xr2:uid="{10B7383D-BFBE-B443-AF96-6E0CFA8FB728}"/>
   </bookViews>
@@ -18,24 +18,26 @@
   <definedNames>
     <definedName name="_xlchart.v1.0" hidden="1">bakery_customers!$F$1</definedName>
     <definedName name="_xlchart.v1.1" hidden="1">bakery_customers!$F$2:$F$51</definedName>
-    <definedName name="_xlchart.v1.10" hidden="1">bakery_customers!$F$1</definedName>
-    <definedName name="_xlchart.v1.11" hidden="1">bakery_customers!$F$2:$F$51</definedName>
+    <definedName name="_xlchart.v1.10" hidden="1">bakery_customers!$E$2:$E$51</definedName>
+    <definedName name="_xlchart.v1.11" hidden="1">bakery_customers!$B$2:$B$51</definedName>
     <definedName name="_xlchart.v1.12" hidden="1">bakery_customers!$E$1</definedName>
     <definedName name="_xlchart.v1.13" hidden="1">bakery_customers!$E$2:$E$51</definedName>
-    <definedName name="_xlchart.v1.14" hidden="1">bakery_customers!$E$1</definedName>
-    <definedName name="_xlchart.v1.15" hidden="1">bakery_customers!$E$2:$E$51</definedName>
-    <definedName name="_xlchart.v1.16" hidden="1">bakery_customers!$E$1</definedName>
-    <definedName name="_xlchart.v1.17" hidden="1">bakery_customers!$E$2:$E$51</definedName>
-    <definedName name="_xlchart.v1.18" hidden="1">bakery_customers!$F$1</definedName>
-    <definedName name="_xlchart.v1.19" hidden="1">bakery_customers!$F$2:$F$51</definedName>
-    <definedName name="_xlchart.v1.2" hidden="1">bakery_customers!$E$1</definedName>
-    <definedName name="_xlchart.v1.3" hidden="1">bakery_customers!$E$2:$E$51</definedName>
-    <definedName name="_xlchart.v1.4" hidden="1">bakery_customers!$F$1</definedName>
-    <definedName name="_xlchart.v1.5" hidden="1">bakery_customers!$F$2:$F$51</definedName>
-    <definedName name="_xlchart.v1.6" hidden="1">bakery_customers!$E$1</definedName>
-    <definedName name="_xlchart.v1.7" hidden="1">bakery_customers!$E$2:$E$51</definedName>
-    <definedName name="_xlchart.v1.8" hidden="1">bakery_customers!$E$1</definedName>
-    <definedName name="_xlchart.v1.9" hidden="1">bakery_customers!$E$2:$E$51</definedName>
+    <definedName name="_xlchart.v1.14" hidden="1">bakery_customers!$B$2:$B$51</definedName>
+    <definedName name="_xlchart.v1.15" hidden="1">bakery_customers!$E$1</definedName>
+    <definedName name="_xlchart.v1.16" hidden="1">bakery_customers!$E$2:$E$51</definedName>
+    <definedName name="_xlchart.v1.17" hidden="1">bakery_customers!$E$1</definedName>
+    <definedName name="_xlchart.v1.18" hidden="1">bakery_customers!$E$2:$E$51</definedName>
+    <definedName name="_xlchart.v1.19" hidden="1">bakery_customers!$B$2:$B$51</definedName>
+    <definedName name="_xlchart.v1.2" hidden="1">bakery_customers!$B$2:$B$51</definedName>
+    <definedName name="_xlchart.v1.20" hidden="1">bakery_customers!$E$1</definedName>
+    <definedName name="_xlchart.v1.21" hidden="1">bakery_customers!$E$2:$E$51</definedName>
+    <definedName name="_xlchart.v1.3" hidden="1">bakery_customers!$E$1</definedName>
+    <definedName name="_xlchart.v1.4" hidden="1">bakery_customers!$E$2:$E$51</definedName>
+    <definedName name="_xlchart.v1.5" hidden="1">bakery_customers!$F$1</definedName>
+    <definedName name="_xlchart.v1.6" hidden="1">bakery_customers!$F$2:$F$51</definedName>
+    <definedName name="_xlchart.v1.7" hidden="1">bakery_customers!$E$1</definedName>
+    <definedName name="_xlchart.v1.8" hidden="1">bakery_customers!$E$2:$E$51</definedName>
+    <definedName name="_xlchart.v1.9" hidden="1">bakery_customers!$E$1</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
@@ -770,7 +772,7 @@
   <cx:chartData>
     <cx:data id="0">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.13</cx:f>
+        <cx:f>_xlchart.v1.8</cx:f>
       </cx:numDim>
     </cx:data>
   </cx:chartData>
@@ -817,7 +819,7 @@
         <cx:series layoutId="clusteredColumn" uniqueId="{00000000-481A-4246-B33F-BF1106AF569E}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.12</cx:f>
+              <cx:f>_xlchart.v1.7</cx:f>
               <cx:v>total_spent_usd</cx:v>
             </cx:txData>
           </cx:tx>
@@ -911,7 +913,7 @@
   <cx:chartData>
     <cx:data id="0">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.11</cx:f>
+        <cx:f>_xlchart.v1.6</cx:f>
       </cx:numDim>
     </cx:data>
   </cx:chartData>
@@ -958,7 +960,7 @@
         <cx:series layoutId="clusteredColumn" uniqueId="{00000000-1CF4-F643-87C9-44A365688FA0}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.10</cx:f>
+              <cx:f>_xlchart.v1.5</cx:f>
               <cx:v>visits_last_year</cx:v>
             </cx:txData>
           </cx:tx>
@@ -1054,7 +1056,7 @@
   <cx:chartData>
     <cx:data id="0">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.15</cx:f>
+        <cx:f>_xlchart.v1.10</cx:f>
       </cx:numDim>
     </cx:data>
   </cx:chartData>
@@ -1101,7 +1103,7 @@
         <cx:series layoutId="boxWhisker" uniqueId="{00000000-7877-1F44-830F-CB2738ACFCD6}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.14</cx:f>
+              <cx:f>_xlchart.v1.9</cx:f>
               <cx:v>total_spent_usd</cx:v>
             </cx:txData>
           </cx:tx>
@@ -1271,6 +1273,142 @@
 </cx:chartSpace>
 </file>
 
+<file path=xl/charts/chartEx5.xml><?xml version="1.0" encoding="utf-8"?>
+<cx:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex">
+  <cx:chartData>
+    <cx:data id="0">
+      <cx:strDim type="cat">
+        <cx:f>_xlchart.v1.14</cx:f>
+      </cx:strDim>
+      <cx:numDim type="val">
+        <cx:f>_xlchart.v1.16</cx:f>
+      </cx:numDim>
+    </cx:data>
+  </cx:chartData>
+  <cx:chart>
+    <cx:title pos="t" align="ctr" overlay="0">
+      <cx:tx>
+        <cx:rich>
+          <a:bodyPr spcFirstLastPara="1" vertOverflow="ellipsis" horzOverflow="overflow" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="ctr" rtl="0">
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US" sz="1400" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                <a:solidFill>
+                  <a:sysClr val="windowText" lastClr="000000">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:sysClr>
+                </a:solidFill>
+                <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+              </a:rPr>
+              <a:t> </a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" sz="1400" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                <a:solidFill>
+                  <a:sysClr val="windowText" lastClr="000000">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:sysClr>
+                </a:solidFill>
+                <a:effectLst/>
+                <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+                <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+                <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              </a:rPr>
+              <a:t>Total Spent by Region</a:t>
+            </a:r>
+            <a:endParaRPr lang="en-US" sz="1400" b="0" i="0" u="none" strike="noStrike" baseline="0">
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:sysClr>
+              </a:solidFill>
+              <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+            </a:endParaRPr>
+          </a:p>
+        </cx:rich>
+      </cx:tx>
+    </cx:title>
+    <cx:plotArea>
+      <cx:plotAreaRegion>
+        <cx:series layoutId="boxWhisker" uniqueId="{00000000-D6FE-5A40-8D73-8BB0E466B388}">
+          <cx:tx>
+            <cx:txData>
+              <cx:f>_xlchart.v1.15</cx:f>
+              <cx:v>total_spent_usd</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:dataId val="0"/>
+          <cx:layoutPr>
+            <cx:visibility meanLine="0" meanMarker="1" nonoutliers="0" outliers="1"/>
+            <cx:statistics quartileMethod="exclusive"/>
+          </cx:layoutPr>
+        </cx:series>
+      </cx:plotAreaRegion>
+      <cx:axis id="0">
+        <cx:catScaling gapWidth="1"/>
+        <cx:tickLabels/>
+      </cx:axis>
+      <cx:axis id="1">
+        <cx:valScaling/>
+        <cx:title>
+          <cx:tx>
+            <cx:rich>
+              <a:bodyPr spcFirstLastPara="1" vertOverflow="ellipsis" horzOverflow="overflow" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr algn="ctr" rtl="0">
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US" sz="900" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                    <a:solidFill>
+                      <a:sysClr val="windowText" lastClr="000000">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:sysClr>
+                    </a:solidFill>
+                    <a:effectLst/>
+                    <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+                    <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+                    <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+                  </a:rPr>
+                  <a:t>Total spent (USD).</a:t>
+                </a:r>
+                <a:endParaRPr lang="en-US" sz="900" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                  <a:solidFill>
+                    <a:sysClr val="windowText" lastClr="000000">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:sysClr>
+                  </a:solidFill>
+                  <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+                </a:endParaRPr>
+              </a:p>
+            </cx:rich>
+          </cx:tx>
+          <cx:extLst>
+            <cx:ext uri="ext:featex">
+              <cx:featureExtension feature="mp" drop="onModelChange">
+                <cx:offset top="-0.1111111119389534"/>
+              </cx:featureExtension>
+            </cx:ext>
+          </cx:extLst>
+        </cx:title>
+        <cx:majorGridlines/>
+        <cx:tickLabels/>
+      </cx:axis>
+    </cx:plotArea>
+  </cx:chart>
+</cx:chartSpace>
+</file>
+
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
@@ -1431,6 +1569,46 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors5.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="366">
   <cs:axisTitle>
@@ -2963,6 +3141,521 @@
 </file>
 
 <file path=xl/charts/style4.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="406">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat">
+        <a:solidFill>
+          <a:srgbClr val="D9D9D9"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDash"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style5.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="406">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
@@ -3791,6 +4484,84 @@
     </mc:AlternateContent>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>673100</xdr:colOff>
+      <xdr:row>48</xdr:row>
+      <xdr:rowOff>57150</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>747183</xdr:colOff>
+      <xdr:row>70</xdr:row>
+      <xdr:rowOff>88900</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" Requires="cx1">
+        <xdr:graphicFrame macro="">
+          <xdr:nvGraphicFramePr>
+            <xdr:cNvPr id="9" name="Chart 8">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{39DAF0EE-943E-C810-8F05-C44DFAB91CC7}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvGraphicFramePr/>
+          </xdr:nvGraphicFramePr>
+          <xdr:xfrm>
+            <a:off x="0" y="0"/>
+            <a:ext cx="0" cy="0"/>
+          </xdr:xfrm>
+          <a:graphic>
+            <a:graphicData uri="http://schemas.microsoft.com/office/drawing/2014/chartex">
+              <cx:chart xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
+            </a:graphicData>
+          </a:graphic>
+        </xdr:graphicFrame>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="0" name=""/>
+            <xdr:cNvSpPr>
+              <a:spLocks noTextEdit="1"/>
+            </xdr:cNvSpPr>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="5626100" y="9810750"/>
+              <a:ext cx="7503583" cy="4502150"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:solidFill>
+              <a:prstClr val="white"/>
+            </a:solidFill>
+            <a:ln w="1">
+              <a:solidFill>
+                <a:prstClr val="green"/>
+              </a:solidFill>
+            </a:ln>
+          </xdr:spPr>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" horzOverflow="clip"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:r>
+                <a:rPr lang="en-US" sz="1100"/>
+                <a:t>This chart isn't available in your version of Excel.
+Editing this shape or saving this workbook into a different file format will permanently break the chart.</a:t>
+              </a:r>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 

</xml_diff>